<commit_message>
added problem for stl
</commit_message>
<xml_diff>
--- a/Course-Outline/Advanced_C-3Days.xlsx
+++ b/Course-Outline/Advanced_C-3Days.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D9DE4F1-59F4-459A-A436-1A12DAB418D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68AFF7E2-A48B-4398-9BB5-BC4586904E30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -359,9 +359,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -383,6 +380,9 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -410,8 +410,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -746,55 +746,55 @@
       <c r="A3" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="10" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="24"/>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="10" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A5" s="24"/>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="10" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="24"/>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="11" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="8"/>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="12" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="8"/>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="15" t="s">
         <v>40</v>
       </c>
     </row>
@@ -809,28 +809,28 @@
       <c r="A10" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="14" t="s">
+      <c r="B10" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="10" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="24"/>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="11" t="s">
+      <c r="C11" s="10" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="25"/>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="11" t="s">
+      <c r="C12" s="10" t="s">
         <v>35</v>
       </c>
     </row>
@@ -845,17 +845,17 @@
       <c r="A14" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="C14" s="16" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="24"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="11" t="s">
+      <c r="B15" s="9"/>
+      <c r="C15" s="10" t="s">
         <v>38</v>
       </c>
     </row>
@@ -897,10 +897,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="26" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>